<commit_message>
Add teacher launcher, portable RunApp data, and full clinic seed data.
Run-ClinicVets.bat for one-click start, SQLite/Excel under RunApp/Data/, and realistic demo records for all main screens.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Source/Data/ClinicVets.xlsx
+++ b/Source/Data/ClinicVets.xlsx
@@ -40,7 +40,7 @@
     <x:t>Role</x:t>
   </x:si>
   <x:si>
-    <x:t>admin1</x:t>
+    <x:t>admin</x:t>
   </x:si>
   <x:si>
     <x:t>1234</x:t>
@@ -58,7 +58,7 @@
     <x:t>Secretary</x:t>
   </x:si>
   <x:si>
-    <x:t>vet123</x:t>
+    <x:t>vet</x:t>
   </x:si>
   <x:si>
     <x:t>0002</x:t>
@@ -73,6 +73,108 @@
     <x:t>Vet</x:t>
   </x:si>
   <x:si>
+    <x:t>jassar1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>#jassar1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jassar@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>213833056</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jassar2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>#j6500sae2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1235</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jassar8521@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>213833058</x:t>
+  </x:si>
+  <x:si>
+    <x:t>sarah1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Pass123!</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1001</x:t>
+  </x:si>
+  <x:si>
+    <x:t>sarah@clinic.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>301234567</x:t>
+  </x:si>
+  <x:si>
+    <x:t>david2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1002</x:t>
+  </x:si>
+  <x:si>
+    <x:t>david@clinic.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>302345678</x:t>
+  </x:si>
+  <x:si>
+    <x:t>noa345</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1003</x:t>
+  </x:si>
+  <x:si>
+    <x:t>noa@clinic.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>303456789</x:t>
+  </x:si>
+  <x:si>
+    <x:t>mike99</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1004</x:t>
+  </x:si>
+  <x:si>
+    <x:t>mike@clinic.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>304567890</x:t>
+  </x:si>
+  <x:si>
+    <x:t>lior12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1005</x:t>
+  </x:si>
+  <x:si>
+    <x:t>lior@clinic.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>305678901</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jassar12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4569</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jasar@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>213833053</x:t>
+  </x:si>
+  <x:si>
     <x:t>IsApproved</x:t>
   </x:si>
   <x:si>
@@ -85,10 +187,34 @@
     <x:t>system</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-06-01T16:43:53.9583098Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-01T16:43:53.9583189Z</x:t>
+    <x:t>2026-06-01T17:13:50.1399736Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-01T17:13:50.1400665Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-01T17:13:50.1400729Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-01T17:13:50.1400780Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-01T17:13:50.1400828Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-01T17:13:50.1400877Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-01T17:13:50.1400921Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-01T17:13:50.1400964Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-01T17:13:50.1401015Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-01T17:13:50.1401058Z</x:t>
   </x:si>
   <x:si>
     <x:t>FullName</x:t>
@@ -529,13 +655,13 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F3"/>
+  <x:dimension ref="A1:F11"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="9.567768" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.710625" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="16.996339" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="17.567768" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="21.567768" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="10.282054" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="9.282054" style="0" customWidth="1"/>
   </x:cols>
@@ -597,6 +723,166 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:6">
+      <x:c r="A4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:6">
+      <x:c r="A5" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:6">
+      <x:c r="A6" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:6">
+      <x:c r="A7" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:6">
+      <x:c r="A8" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:6">
+      <x:c r="A9" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:6">
+      <x:c r="A10" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="F10" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:6">
+      <x:c r="A11" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F11" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
     </x:row>
@@ -614,7 +900,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D3"/>
+  <x:dimension ref="A1:D11"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
@@ -628,13 +914,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4">
@@ -645,10 +931,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:4">
@@ -659,10 +945,122 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>56</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:4">
+      <x:c r="A4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B4" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:4">
+      <x:c r="A5" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B5" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:4">
+      <x:c r="A6" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B6" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:4">
+      <x:c r="A7" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B7" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:4">
+      <x:c r="A8" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B8" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:4">
+      <x:c r="A9" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B9" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:4">
+      <x:c r="A10" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B10" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:4">
+      <x:c r="A11" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B11" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>64</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -694,16 +1092,16 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -735,28 +1133,28 @@
   <x:sheetData>
     <x:row r="1" spans="1:8">
       <x:c r="A1" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -786,22 +1184,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -838,43 +1236,43 @@
   <x:sheetData>
     <x:row r="1" spans="1:13">
       <x:c r="A1" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="I1" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="J1" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="K1" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="L1" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="M1" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -904,22 +1302,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add login AuthService with functional tests and refresh demo seed
Extract login logic from LoginView into testable AuthService.TryLogin returning a LoginResult (success, error, employee, role, reason). Add 10 login functional tests covering valid/invalid/empty/pending/rejected and role checks. Align demo seed accounts (admin1, EmployeeNumbers 1001-1006) and rebuild RunApp publish output and demo Excel mirror.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Source/Data/ClinicVets.xlsx
+++ b/Source/Data/ClinicVets.xlsx
@@ -40,73 +40,64 @@
     <x:t>Role</x:t>
   </x:si>
   <x:si>
-    <x:t>admin</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1234</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0001</x:t>
+    <x:t>admin1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Admin123!</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1001</x:t>
   </x:si>
   <x:si>
     <x:t>admin@clinic.com</x:t>
   </x:si>
   <x:si>
-    <x:t>000000001</x:t>
+    <x:t>300000018</x:t>
   </x:si>
   <x:si>
     <x:t>Secretary</x:t>
   </x:si>
   <x:si>
-    <x:t>vet</x:t>
-  </x:si>
-  <x:si>
-    <x:t>0002</x:t>
+    <x:t>secuser</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sec123!a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1002</x:t>
+  </x:si>
+  <x:si>
+    <x:t>sec@clinic.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>300000027</x:t>
+  </x:si>
+  <x:si>
+    <x:t>vetuser</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Vet123!a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1003</x:t>
   </x:si>
   <x:si>
     <x:t>vet@clinic.com</x:t>
   </x:si>
   <x:si>
-    <x:t>000000002</x:t>
+    <x:t>300000036</x:t>
   </x:si>
   <x:si>
     <x:t>Vet</x:t>
   </x:si>
   <x:si>
-    <x:t>jassar1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>#jassar1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>jassar@gmail.com</x:t>
-  </x:si>
-  <x:si>
-    <x:t>213833056</x:t>
-  </x:si>
-  <x:si>
-    <x:t>jassar2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>#j6500sae2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1235</x:t>
-  </x:si>
-  <x:si>
-    <x:t>jassar8521@gmail.com</x:t>
-  </x:si>
-  <x:si>
-    <x:t>213833058</x:t>
-  </x:si>
-  <x:si>
     <x:t>sarah1</x:t>
   </x:si>
   <x:si>
     <x:t>Pass123!</x:t>
   </x:si>
   <x:si>
-    <x:t>1001</x:t>
+    <x:t>1004</x:t>
   </x:si>
   <x:si>
     <x:t>sarah@clinic.com</x:t>
@@ -118,7 +109,7 @@
     <x:t>david2</x:t>
   </x:si>
   <x:si>
-    <x:t>1002</x:t>
+    <x:t>1005</x:t>
   </x:si>
   <x:si>
     <x:t>david@clinic.com</x:t>
@@ -127,54 +118,18 @@
     <x:t>302345678</x:t>
   </x:si>
   <x:si>
-    <x:t>noa345</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1003</x:t>
-  </x:si>
-  <x:si>
-    <x:t>noa@clinic.com</x:t>
+    <x:t>roni12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1006</x:t>
+  </x:si>
+  <x:si>
+    <x:t>roni@clinic.com</x:t>
   </x:si>
   <x:si>
     <x:t>303456789</x:t>
   </x:si>
   <x:si>
-    <x:t>mike99</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1004</x:t>
-  </x:si>
-  <x:si>
-    <x:t>mike@clinic.com</x:t>
-  </x:si>
-  <x:si>
-    <x:t>304567890</x:t>
-  </x:si>
-  <x:si>
-    <x:t>lior12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1005</x:t>
-  </x:si>
-  <x:si>
-    <x:t>lior@clinic.com</x:t>
-  </x:si>
-  <x:si>
-    <x:t>305678901</x:t>
-  </x:si>
-  <x:si>
-    <x:t>jassar12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4569</x:t>
-  </x:si>
-  <x:si>
-    <x:t>jasar@gmail.com</x:t>
-  </x:si>
-  <x:si>
-    <x:t>213833053</x:t>
-  </x:si>
-  <x:si>
     <x:t>IsApproved</x:t>
   </x:si>
   <x:si>
@@ -187,34 +142,22 @@
     <x:t>system</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-06-01T17:13:50.1399736Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-01T17:13:50.1400665Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-01T17:13:50.1400729Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-01T17:13:50.1400780Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-01T17:13:50.1400828Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-01T17:13:50.1400877Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-01T17:13:50.1400921Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-01T17:13:50.1400964Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-01T17:13:50.1401015Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-01T17:13:50.1401058Z</x:t>
+    <x:t>2026-06-14T11:20:23.5659675Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T11:20:23.5659884Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T11:20:23.5660013Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T11:20:23.5660141Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T11:20:23.5660274Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T11:20:23.5660401Z</x:t>
   </x:si>
   <x:si>
     <x:t>FullName</x:t>
@@ -226,6 +169,72 @@
     <x:t>Gender</x:t>
   </x:si>
   <x:si>
+    <x:t>123456782</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Fares Mansour</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0501234567</x:t>
+  </x:si>
+  <x:si>
+    <x:t>fares@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>זכר</x:t>
+  </x:si>
+  <x:si>
+    <x:t>234567891</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Maya Levi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0529876543</x:t>
+  </x:si>
+  <x:si>
+    <x:t>maya@example.co.il</x:t>
+  </x:si>
+  <x:si>
+    <x:t>נקבה</x:t>
+  </x:si>
+  <x:si>
+    <x:t>345678902</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Yosef Cohen</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0541112233</x:t>
+  </x:si>
+  <x:si>
+    <x:t>yosef@company.org</x:t>
+  </x:si>
+  <x:si>
+    <x:t>456789013</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Dana Shapiro</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0534445566</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dana@site.net</x:t>
+  </x:si>
+  <x:si>
+    <x:t>567890124</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ron Azulay</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0509988776</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ron@clinic.com</x:t>
+  </x:si>
+  <x:si>
     <x:t>Id</x:t>
   </x:si>
   <x:si>
@@ -250,6 +259,90 @@
     <x:t>LastVaccinationDate</x:t>
   </x:si>
   <x:si>
+    <x:t>ZAZA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>כלב</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3761234</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2020-03-15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2025-10-14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Mitzi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>חתול</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3762345</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2021-07-20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-03-14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Rio</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ציפור</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3763456</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2022-01-10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2025-07-14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Spike</x:t>
+  </x:si>
+  <x:si>
+    <x:t>זוחל</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3764567</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2019-11-05</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2025-04-14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Buddy</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3765678</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2018-05-22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-05-25</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Luna</x:t>
+  </x:si>
+  <x:si>
+    <x:t>3766789</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2023-02-08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-05-14</x:t>
+  </x:si>
+  <x:si>
     <x:t>StockQuantity</x:t>
   </x:si>
   <x:si>
@@ -262,6 +355,60 @@
     <x:t>Notes</x:t>
   </x:si>
   <x:si>
+    <x:t>Antibiotic</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2027-04-14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>שגרתי למסלול טיפול</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Pain Relief</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-12-14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>לאחר ניתוח</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Rabies Vaccine</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2027-06-14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>חיסון שנתי</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Flea Drops</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2027-02-14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>טיפול חיצוני</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Vitamin Complex</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2027-08-14</x:t>
+  </x:si>
+  <x:si>
+    <x:t>תוסף תזונה</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ear Drops</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-07-29</x:t>
+  </x:si>
+  <x:si>
+    <x:t>דורש מעקב מלאי</x:t>
+  </x:si>
+  <x:si>
     <x:t>AnimalChipNumber</x:t>
   </x:si>
   <x:si>
@@ -296,6 +443,75 @@
   </x:si>
   <x:si>
     <x:t>ArrivalNote</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-18 10:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Vaccination</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>Annual rabies booster</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scheduled</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-09 11:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Checkup</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Reported by owner</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Routine wellness exam</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Arrived</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-16 09:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Wing trim</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Scheduled grooming visit</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-02 14:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Skin issue</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Antibiotic course for infection</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-13 16:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Limping</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Owner did not arrive</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NoShow</x:t>
+  </x:si>
+  <x:si>
+    <x:t>לא הגיע לתור</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14 15:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Flea prevention treatment</x:t>
   </x:si>
   <x:si>
     <x:t>VisitId</x:t>
@@ -655,13 +871,13 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F11"/>
+  <x:dimension ref="A1:F7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.567768" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="16.996339" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="21.567768" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.567768" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="10.282054" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="9.282054" style="0" customWidth="1"/>
   </x:cols>
@@ -711,19 +927,19 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -734,33 +950,33 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:6">
       <x:c r="A5" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
         <x:v>11</x:v>
@@ -768,122 +984,42 @@
     </x:row>
     <x:row r="6" spans="1:6">
       <x:c r="A6" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:6">
       <x:c r="A7" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:6">
-      <x:c r="A8" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="D8" s="0" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="E8" s="0" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="F8" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:6">
-      <x:c r="A9" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="C9" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="D9" s="0" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="E9" s="0" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="F9" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:6">
-      <x:c r="A10" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="C10" s="0" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D10" s="0" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="E10" s="0" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="F10" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:6">
-      <x:c r="A11" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="B11" s="0" t="s">
         <x:v>22</x:v>
-      </x:c>
-      <x:c r="C11" s="0" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="D11" s="0" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="E11" s="0" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="F11" s="0" t="s">
-        <x:v>16</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -900,7 +1036,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D11"/>
+  <x:dimension ref="A1:D7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
@@ -914,13 +1050,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4">
@@ -931,10 +1067,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:4">
@@ -945,10 +1081,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:4">
@@ -959,108 +1095,52 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>42</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:4">
       <x:c r="A5" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B5" s="0">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:4">
       <x:c r="A6" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B6" s="0">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:4">
       <x:c r="A7" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B7" s="0">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:4">
-      <x:c r="A8" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B8" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="D8" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:4">
-      <x:c r="A9" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="B9" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C9" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="D9" s="0" t="s">
-        <x:v>62</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:4">
-      <x:c r="A10" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="B10" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C10" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="D10" s="0" t="s">
-        <x:v>63</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:4">
-      <x:c r="A11" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="B11" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C11" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="D11" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>45</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1077,13 +1157,13 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:E1"/>
+  <x:dimension ref="A1:E6"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="9.282054" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="6.567768" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="5.567768" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="10.282054" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14.424911" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11.282054" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19.710625" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="7.567768" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -1092,16 +1172,101 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:5">
+      <x:c r="A2" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:5">
+      <x:c r="A3" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:5">
+      <x:c r="A4" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:5">
+      <x:c r="A5" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:5">
+      <x:c r="A6" s="0" t="s">
         <x:v>67</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>53</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1118,43 +1283,199 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:H1"/>
+  <x:dimension ref="A1:H7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="2.710625" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="5.996339" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="6.567768" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="7.567768" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="12.424911" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="7.424911" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.424911" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="10.424911" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="15.996339" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="19.139196" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:8">
       <x:c r="A1" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>78</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:8">
+      <x:c r="A2" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="E2" s="0">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:8">
+      <x:c r="A3" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="E3" s="0">
+        <x:v>4.2</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:8">
+      <x:c r="A4" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="E4" s="0">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="s">
+        <x:v>93</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:8">
+      <x:c r="A5" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="E5" s="0">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H5" s="0" t="s">
+        <x:v>98</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:8">
+      <x:c r="A6" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E6" s="0">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="H6" s="0" t="s">
+        <x:v>102</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:8">
+      <x:c r="A7" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="E7" s="0">
+        <x:v>3.9</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="H7" s="0" t="s">
+        <x:v>106</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1171,35 +1492,155 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F1"/>
+  <x:dimension ref="A1:F7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="2.710625" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="5.996339" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15.996339" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="13.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="8.996339" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="14.139196" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="5.996339" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>110</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:6">
+      <x:c r="A2" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="C2" s="0">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="D2" s="0">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>113</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:6">
+      <x:c r="A3" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="C3" s="0">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D3" s="0">
+        <x:v>18.5</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>116</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:6">
+      <x:c r="A4" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="C4" s="0">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D4" s="0">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>119</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:6">
+      <x:c r="A5" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="C5" s="0">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D5" s="0">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>122</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:6">
+      <x:c r="A6" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="C6" s="0">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D6" s="0">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:6">
+      <x:c r="A7" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="C7" s="0">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D7" s="0">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>128</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1216,63 +1657,309 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:M1"/>
+  <x:dimension ref="A1:M7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="2.710625" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="18.567768" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="8.853482" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="7.567768" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="10.567768" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="9.424911" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15.710625" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11.139196" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18.282054" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="27.139196" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="16.996339" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="9.139196" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="16.282054" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="19.139196" style="0" customWidth="1"/>
     <x:col min="11" max="11" width="9.424911" style="0" customWidth="1"/>
     <x:col min="12" max="12" width="12.424911" style="0" customWidth="1"/>
-    <x:col min="13" max="13" width="10.853482" style="0" customWidth="1"/>
+    <x:col min="13" max="13" width="11.139196" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:13">
       <x:c r="A1" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="C1" s="0" t="s">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="D1" s="0" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="E1" s="0" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F1" s="0" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="G1" s="0" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="H1" s="0" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="I1" s="0" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="J1" s="0" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="K1" s="0" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="L1" s="0" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="M1" s="0" t="s">
+        <x:v>140</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:13">
+      <x:c r="A2" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H2" s="0">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="I2" s="0" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="J2" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K2" s="0">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="L2" s="0" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="M2" s="0" t="s">
+        <x:v>143</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:13">
+      <x:c r="A3" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H3" s="0">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="I3" s="0" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="J3" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K3" s="0">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="L3" s="0" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="M3" s="0" t="s">
+        <x:v>143</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:13">
+      <x:c r="A4" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H4" s="0">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="C1" s="0" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="D1" s="0" t="s">
-        <x:v>82</x:v>
-      </x:c>
-      <x:c r="E1" s="0" t="s">
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="F1" s="0" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="G1" s="0" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="H1" s="0" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="I1" s="0" t="s">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="J1" s="0" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="K1" s="0" t="s">
-        <x:v>89</x:v>
-      </x:c>
-      <x:c r="L1" s="0" t="s">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="M1" s="0" t="s">
-        <x:v>91</x:v>
+      <x:c r="I4" s="0" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="J4" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K4" s="0">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="L4" s="0" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="M4" s="0" t="s">
+        <x:v>143</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:13">
+      <x:c r="A5" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H5" s="0">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="I5" s="0" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="J5" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K5" s="0">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="L5" s="0" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="M5" s="0" t="s">
+        <x:v>143</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:13">
+      <x:c r="A6" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H6" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I6" s="0" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="J6" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K6" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L6" s="0" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="M6" s="0" t="s">
+        <x:v>161</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:13">
+      <x:c r="A7" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H7" s="0">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I7" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="J7" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K7" s="0">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="L7" s="0" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="M7" s="0" t="s">
+        <x:v>143</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1289,12 +1976,12 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F1"/>
+  <x:dimension ref="A1:F7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="2.710625" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="6.282054" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="10.996339" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="27.139196" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="16.282054" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="19.139196" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="8.567768" style="0" customWidth="1"/>
@@ -1302,22 +1989,142 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>166</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:6">
+      <x:c r="A2" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="E2" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="0">
+        <x:v>95</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:6">
+      <x:c r="A3" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="E3" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F3" s="0">
+        <x:v>24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:6">
+      <x:c r="A4" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="E4" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F4" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:6">
+      <x:c r="A5" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="E5" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F5" s="0">
+        <x:v>75</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:6">
+      <x:c r="A6" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B6" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="E6" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:6">
+      <x:c r="A7" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B7" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="E7" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F7" s="0">
+        <x:v>42</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Final project update: demo data, validations, tests, UI improvements, and documentation
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Source/Data/ClinicVets.xlsx
+++ b/Source/Data/ClinicVets.xlsx
@@ -142,22 +142,22 @@
     <x:t>system</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-06-14T11:20:23.5659675Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T11:20:23.5659884Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T11:20:23.5660013Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T11:20:23.5660141Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T11:20:23.5660274Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T11:20:23.5660401Z</x:t>
+    <x:t>2026-06-14T11:55:33.8042375Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T11:55:33.8042739Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T11:55:33.8042786Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T11:55:33.8042843Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T11:55:33.8042901Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T11:55:33.8042942Z</x:t>
   </x:si>
   <x:si>
     <x:t>FullName</x:t>

</xml_diff>

<commit_message>
Remove employee approval system
Delete the vestigial employee-approval feature that the project no longer needs:

- Drop IsApproved from the Employee model and the EmployeeApprovals SQLite table (with a DROP migration so existing DBs stay consistent) and the EmployeeApprovals Excel sheet.

- Remove the not-approved check/reason/message from AuthService and LoginView so login works immediately after registration.

- Registration creates a normal employee directly; Employee ID stays 4-digit unique, roles remain Secretary/Veterinarian.

- Update demo seed data and tests (drop approval-only fixtures/tests, assert the EmployeeApprovals sheet is absent). All 60 tests pass.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Source/Data/ClinicVets.xlsx
+++ b/Source/Data/ClinicVets.xlsx
@@ -7,12 +7,11 @@
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Employees" sheetId="1" r:id="rId2"/>
-    <x:sheet name="EmployeeApprovals" sheetId="2" r:id="rId3"/>
-    <x:sheet name="Clients" sheetId="3" r:id="rId4"/>
-    <x:sheet name="Animals" sheetId="4" r:id="rId5"/>
-    <x:sheet name="Medications" sheetId="5" r:id="rId6"/>
-    <x:sheet name="Visits" sheetId="6" r:id="rId7"/>
-    <x:sheet name="Treatments" sheetId="7" r:id="rId8"/>
+    <x:sheet name="Clients" sheetId="2" r:id="rId3"/>
+    <x:sheet name="Animals" sheetId="3" r:id="rId4"/>
+    <x:sheet name="Medications" sheetId="4" r:id="rId5"/>
+    <x:sheet name="Visits" sheetId="5" r:id="rId6"/>
+    <x:sheet name="Treatments" sheetId="6" r:id="rId7"/>
   </x:sheets>
   <x:definedNames/>
   <x:calcPr calcId="125725"/>
@@ -128,36 +127,6 @@
   </x:si>
   <x:si>
     <x:t>303456789</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IsApproved</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ApprovedBy</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ApprovedAt</x:t>
-  </x:si>
-  <x:si>
-    <x:t>system</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T11:55:33.8042375Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T11:55:33.8042739Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T11:55:33.8042786Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T11:55:33.8042843Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T11:55:33.8042901Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T11:55:33.8042942Z</x:t>
   </x:si>
   <x:si>
     <x:t>FullName</x:t>
@@ -1036,127 +1005,6 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D7"/>
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="11.139196" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="11.853482" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="28.282054" style="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" spans="1:4">
-      <x:c r="A1" s="0" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B1" s="0" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="C1" s="0" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="D1" s="0" t="s">
-        <x:v>38</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:4">
-      <x:c r="A2" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B2" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C2" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D2" s="0" t="s">
-        <x:v>40</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:4">
-      <x:c r="A3" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B3" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>41</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:4">
-      <x:c r="A4" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B4" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>42</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:4">
-      <x:c r="A5" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="B5" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D5" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:4">
-      <x:c r="A6" s="0" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="B6" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D6" s="0" t="s">
-        <x:v>44</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:4">
-      <x:c r="A7" s="0" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B7" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D7" s="0" t="s">
-        <x:v>45</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
-  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
-  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
-  <x:headerFooter/>
-  <x:tableParts count="0"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <x:sheetPr>
-    <x:outlinePr summaryBelow="1" summaryRight="1"/>
-  </x:sheetPr>
   <x:dimension ref="A1:E6"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1172,101 +1020,101 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5">
       <x:c r="A2" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5">
       <x:c r="A3" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
       <x:c r="A5" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5">
       <x:c r="A6" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1278,7 +1126,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1298,28 +1146,28 @@
   <x:sheetData>
     <x:row r="1" spans="1:8">
       <x:c r="A1" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>68</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:8">
@@ -1327,25 +1175,25 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>12.5</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:8">
@@ -1353,25 +1201,25 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E3" s="0">
         <x:v>4.2</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="H3" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:8">
@@ -1379,25 +1227,25 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="H4" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:8">
@@ -1405,25 +1253,25 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="E5" s="0">
         <x:v>1.8</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="H5" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:8">
@@ -1431,25 +1279,25 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E6" s="0">
         <x:v>28</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="H6" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:8">
@@ -1457,25 +1305,25 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="E7" s="0">
         <x:v>3.9</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="G7" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="H7" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1487,7 +1335,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1505,22 +1353,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1528,7 +1376,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C2" s="0">
         <x:v>45</x:v>
@@ -1537,10 +1385,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1548,7 +1396,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="C3" s="0">
         <x:v>30</x:v>
@@ -1557,10 +1405,10 @@
         <x:v>18.5</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1568,7 +1416,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="C4" s="0">
         <x:v>20</x:v>
@@ -1577,10 +1425,10 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>118</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:6">
@@ -1588,7 +1436,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>120</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C5" s="0">
         <x:v>25</x:v>
@@ -1597,10 +1445,10 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>121</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>122</x:v>
+        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:6">
@@ -1608,7 +1456,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>123</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C6" s="0">
         <x:v>50</x:v>
@@ -1617,10 +1465,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:6">
@@ -1628,7 +1476,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>126</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="C7" s="0">
         <x:v>15</x:v>
@@ -1637,10 +1485,10 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>127</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>128</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1652,7 +1500,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1677,43 +1525,43 @@
   <x:sheetData>
     <x:row r="1" spans="1:13">
       <x:c r="A1" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="C1" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="D1" s="0" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="E1" s="0" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F1" s="0" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="G1" s="0" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="H1" s="0" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="I1" s="0" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="J1" s="0" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="K1" s="0" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="L1" s="0" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="C1" s="0" t="s">
+      <x:c r="M1" s="0" t="s">
         <x:v>130</x:v>
-      </x:c>
-      <x:c r="D1" s="0" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="E1" s="0" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="F1" s="0" t="s">
-        <x:v>133</x:v>
-      </x:c>
-      <x:c r="G1" s="0" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="H1" s="0" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="I1" s="0" t="s">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="J1" s="0" t="s">
-        <x:v>137</x:v>
-      </x:c>
-      <x:c r="K1" s="0" t="s">
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="L1" s="0" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="M1" s="0" t="s">
-        <x:v>140</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:13">
@@ -1721,19 +1569,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>141</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>142</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>144</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
         <x:v>17</x:v>
@@ -1742,7 +1590,7 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="J2" s="0">
         <x:v>1</x:v>
@@ -1751,10 +1599,10 @@
         <x:v>215</x:v>
       </x:c>
       <x:c r="L2" s="0" t="s">
-        <x:v>145</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="M2" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:13">
@@ -1762,19 +1610,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>146</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>147</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
         <x:v>17</x:v>
@@ -1783,7 +1631,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="I3" s="0" t="s">
-        <x:v>123</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="J3" s="0">
         <x:v>2</x:v>
@@ -1792,10 +1640,10 @@
         <x:v>114</x:v>
       </x:c>
       <x:c r="L3" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="M3" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:13">
@@ -1803,19 +1651,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>151</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>152</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
         <x:v>143</x:v>
-      </x:c>
-      <x:c r="F4" s="0" t="s">
-        <x:v>153</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
         <x:v>17</x:v>
@@ -1824,7 +1672,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="I4" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="J4" s="0">
         <x:v>0</x:v>
@@ -1833,10 +1681,10 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="L4" s="0" t="s">
-        <x:v>145</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="M4" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:13">
@@ -1844,19 +1692,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>154</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>155</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>156</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
         <x:v>17</x:v>
@@ -1865,7 +1713,7 @@
         <x:v>110</x:v>
       </x:c>
       <x:c r="I5" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="J5" s="0">
         <x:v>3</x:v>
@@ -1874,10 +1722,10 @@
         <x:v>185</x:v>
       </x:c>
       <x:c r="L5" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="M5" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:13">
@@ -1885,19 +1733,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>157</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>158</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>159</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
         <x:v>17</x:v>
@@ -1906,7 +1754,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="J6" s="0">
         <x:v>0</x:v>
@@ -1915,10 +1763,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L6" s="0" t="s">
-        <x:v>160</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M6" s="0" t="s">
-        <x:v>161</x:v>
+        <x:v>151</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:13">
@@ -1926,19 +1774,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>162</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>142</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>163</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="G7" s="0" t="s">
         <x:v>17</x:v>
@@ -1947,7 +1795,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="I7" s="0" t="s">
-        <x:v>120</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="J7" s="0">
         <x:v>1</x:v>
@@ -1956,10 +1804,10 @@
         <x:v>142</x:v>
       </x:c>
       <x:c r="L7" s="0" t="s">
-        <x:v>145</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="M7" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1971,7 +1819,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1989,22 +1837,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>164</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>165</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>166</x:v>
+        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -2015,10 +1863,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>144</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>1</x:v>
@@ -2035,10 +1883,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>123</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E3" s="0">
         <x:v>2</x:v>
@@ -2055,10 +1903,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>0</x:v>
@@ -2075,10 +1923,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>156</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="E5" s="0">
         <x:v>3</x:v>
@@ -2095,10 +1943,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>159</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="E6" s="0">
         <x:v>0</x:v>
@@ -2115,10 +1963,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>163</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>120</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E7" s="0">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Refresh demo Excel mirror
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Source/Data/ClinicVets.xlsx
+++ b/Source/Data/ClinicVets.xlsx
@@ -7,11 +7,12 @@
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Employees" sheetId="1" r:id="rId2"/>
-    <x:sheet name="Clients" sheetId="2" r:id="rId3"/>
-    <x:sheet name="Animals" sheetId="3" r:id="rId4"/>
-    <x:sheet name="Medications" sheetId="4" r:id="rId5"/>
-    <x:sheet name="Visits" sheetId="5" r:id="rId6"/>
-    <x:sheet name="Treatments" sheetId="6" r:id="rId7"/>
+    <x:sheet name="EmployeeApprovals" sheetId="2" r:id="rId3"/>
+    <x:sheet name="Clients" sheetId="3" r:id="rId4"/>
+    <x:sheet name="Animals" sheetId="4" r:id="rId5"/>
+    <x:sheet name="Medications" sheetId="5" r:id="rId6"/>
+    <x:sheet name="Visits" sheetId="6" r:id="rId7"/>
+    <x:sheet name="Treatments" sheetId="7" r:id="rId8"/>
   </x:sheets>
   <x:definedNames/>
   <x:calcPr calcId="125725"/>
@@ -127,6 +128,54 @@
   </x:si>
   <x:si>
     <x:t>303456789</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jassar</x:t>
+  </x:si>
+  <x:si>
+    <x:t>#Jassar1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1234</x:t>
+  </x:si>
+  <x:si>
+    <x:t>jassar8520@gmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t>213833056</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IsApproved</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ApprovedBy</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ApprovedAt</x:t>
+  </x:si>
+  <x:si>
+    <x:t>system</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T13:02:46.6301001Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T13:02:46.6301232Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T13:02:46.6301277Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T13:02:46.6301331Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T13:02:46.6301369Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T13:02:46.6301403Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T13:02:46.6301447Z</x:t>
   </x:si>
   <x:si>
     <x:t>FullName</x:t>
@@ -840,13 +889,13 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F7"/>
+  <x:dimension ref="A1:F8"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="10.567768" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="16.996339" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="17.567768" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="21.567768" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="10.282054" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="9.282054" style="0" customWidth="1"/>
   </x:cols>
@@ -988,6 +1037,26 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:6">
+      <x:c r="A8" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
     </x:row>
@@ -1001,6 +1070,141 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:D8"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.139196" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11.853482" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28.282054" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:4">
+      <x:c r="A1" s="0" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C1" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D1" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:4">
+      <x:c r="A2" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B2" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:4">
+      <x:c r="A3" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B3" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:4">
+      <x:c r="A4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B4" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:4">
+      <x:c r="A5" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B5" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:4">
+      <x:c r="A6" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B6" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:4">
+      <x:c r="A7" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B7" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:4">
+      <x:c r="A8" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B8" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1020,101 +1224,101 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
         <x:v>3</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>54</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5">
       <x:c r="A2" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5">
       <x:c r="A3" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
       <x:c r="A5" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5">
       <x:c r="A6" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
         <x:v>59</x:v>
-      </x:c>
-      <x:c r="D6" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="E6" s="0" t="s">
-        <x:v>43</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1126,7 +1330,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1146,28 +1350,28 @@
   <x:sheetData>
     <x:row r="1" spans="1:8">
       <x:c r="A1" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:8">
@@ -1175,25 +1379,25 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>12.5</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:8">
@@ -1201,25 +1405,25 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="E3" s="0">
         <x:v>4.2</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="H3" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:8">
@@ -1227,25 +1431,25 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="H4" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:8">
@@ -1253,25 +1457,25 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="E5" s="0">
         <x:v>1.8</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="H5" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>104</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:8">
@@ -1279,25 +1483,25 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="E6" s="0">
         <x:v>28</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="H6" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:8">
@@ -1305,25 +1509,25 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E7" s="0">
         <x:v>3.9</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="G7" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H7" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>112</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1335,7 +1539,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1353,22 +1557,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1376,7 +1580,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="C2" s="0">
         <x:v>45</x:v>
@@ -1385,10 +1589,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>119</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1396,7 +1600,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C3" s="0">
         <x:v>30</x:v>
@@ -1405,10 +1609,10 @@
         <x:v>18.5</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>122</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1416,7 +1620,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="C4" s="0">
         <x:v>20</x:v>
@@ -1425,10 +1629,10 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>125</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:6">
@@ -1436,7 +1640,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C5" s="0">
         <x:v>25</x:v>
@@ -1445,10 +1649,10 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:6">
@@ -1456,7 +1660,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="C6" s="0">
         <x:v>50</x:v>
@@ -1465,10 +1669,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>131</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:6">
@@ -1476,7 +1680,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C7" s="0">
         <x:v>15</x:v>
@@ -1485,10 +1689,10 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>118</x:v>
+        <x:v>134</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1500,7 +1704,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1525,43 +1729,43 @@
   <x:sheetData>
     <x:row r="1" spans="1:13">
       <x:c r="A1" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>120</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>121</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>122</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>123</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="I1" s="0" t="s">
-        <x:v>126</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="J1" s="0" t="s">
-        <x:v>127</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="K1" s="0" t="s">
-        <x:v>128</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="L1" s="0" t="s">
-        <x:v>129</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="M1" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>146</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:13">
@@ -1569,19 +1773,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>131</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>132</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>134</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
         <x:v>17</x:v>
@@ -1590,7 +1794,7 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="J2" s="0">
         <x:v>1</x:v>
@@ -1599,10 +1803,10 @@
         <x:v>215</x:v>
       </x:c>
       <x:c r="L2" s="0" t="s">
-        <x:v>135</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="M2" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>149</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:13">
@@ -1610,19 +1814,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>138</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>139</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
         <x:v>17</x:v>
@@ -1631,7 +1835,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="I3" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="J3" s="0">
         <x:v>2</x:v>
@@ -1640,10 +1844,10 @@
         <x:v>114</x:v>
       </x:c>
       <x:c r="L3" s="0" t="s">
-        <x:v>140</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="M3" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>149</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:13">
@@ -1651,19 +1855,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>141</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>142</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
         <x:v>17</x:v>
@@ -1672,7 +1876,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="I4" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="J4" s="0">
         <x:v>0</x:v>
@@ -1681,10 +1885,10 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="L4" s="0" t="s">
-        <x:v>135</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="M4" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>149</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:13">
@@ -1692,19 +1896,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>144</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>145</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>138</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>146</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
         <x:v>17</x:v>
@@ -1713,7 +1917,7 @@
         <x:v>110</x:v>
       </x:c>
       <x:c r="I5" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="J5" s="0">
         <x:v>3</x:v>
@@ -1722,10 +1926,10 @@
         <x:v>185</x:v>
       </x:c>
       <x:c r="L5" s="0" t="s">
-        <x:v>140</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="M5" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>149</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:13">
@@ -1733,19 +1937,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>147</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>138</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
         <x:v>17</x:v>
@@ -1754,7 +1958,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="J6" s="0">
         <x:v>0</x:v>
@@ -1763,10 +1967,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L6" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="M6" s="0" t="s">
-        <x:v>151</x:v>
+        <x:v>167</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:13">
@@ -1774,19 +1978,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>152</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>132</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="G7" s="0" t="s">
         <x:v>17</x:v>
@@ -1795,7 +1999,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="I7" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="J7" s="0">
         <x:v>1</x:v>
@@ -1804,10 +2008,10 @@
         <x:v>142</x:v>
       </x:c>
       <x:c r="L7" s="0" t="s">
-        <x:v>135</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="M7" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>149</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1819,7 +2023,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1837,22 +2041,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>154</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>155</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>126</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>127</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>156</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1863,10 +2067,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>134</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>1</x:v>
@@ -1883,10 +2087,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>139</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E3" s="0">
         <x:v>2</x:v>
@@ -1903,10 +2107,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>0</x:v>
@@ -1923,10 +2127,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>146</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="E5" s="0">
         <x:v>3</x:v>
@@ -1943,10 +2147,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
         <x:v>149</x:v>
-      </x:c>
-      <x:c r="D6" s="0" t="s">
-        <x:v>133</x:v>
       </x:c>
       <x:c r="E6" s="0">
         <x:v>0</x:v>
@@ -1963,10 +2167,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="E7" s="0">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Show latest vet note on animal card/details
Surface the most recent veterinarian note (Visit.ArrivalNote) on the animal card, the animal edit form, and the visits-screen animal panel by deriving it from the animal's visits via a new AnimalNoteService. The note refreshes immediately after saving a visit and persists across restarts since it is read from already-persisted visit data. Includes unit tests.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Source/Data/ClinicVets.xlsx
+++ b/Source/Data/ClinicVets.xlsx
@@ -157,25 +157,25 @@
     <x:t>system</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-06-14T13:02:46.6301001Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T13:02:46.6301232Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T13:02:46.6301277Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T13:02:46.6301331Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T13:02:46.6301369Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T13:02:46.6301403Z</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-14T13:02:46.6301447Z</x:t>
+    <x:t>2026-06-14T17:52:13.5182800Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T17:52:13.5182870Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T17:52:13.5182922Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T17:52:13.5182970Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T17:52:13.5183023Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T17:52:13.5183068Z</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-14T17:52:13.5183114Z</x:t>
   </x:si>
   <x:si>
     <x:t>FullName</x:t>
@@ -319,7 +319,7 @@
     <x:t>2022-01-10</x:t>
   </x:si>
   <x:si>
-    <x:t>2025-07-14</x:t>
+    <x:t>2024-07-14</x:t>
   </x:si>
   <x:si>
     <x:t>Spike</x:t>
@@ -376,7 +376,7 @@
     <x:t>Antibiotic</x:t>
   </x:si>
   <x:si>
-    <x:t>2027-04-14</x:t>
+    <x:t>2028-04-14</x:t>
   </x:si>
   <x:si>
     <x:t>שגרתי למסלול טיפול</x:t>
@@ -539,6 +539,12 @@
   </x:si>
   <x:si>
     <x:t>LineCost</x:t>
+  </x:si>
+  <x:si>
+    <x:t>תרופה</x:t>
+  </x:si>
+  <x:si>
+    <x:t>צריך חיסון מיידי</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1547,7 +1553,7 @@
   <x:dimension ref="A1:F7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="2.710625" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="2.996339" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="15.996339" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="13.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="8.996339" style="0" customWidth="1"/>
@@ -1577,13 +1583,13 @@
     </x:row>
     <x:row r="2" spans="1:6">
       <x:c r="A2" s="0">
-        <x:v>1</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>117</x:v>
       </x:c>
       <x:c r="C2" s="0">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D2" s="0">
         <x:v>25</x:v>
@@ -1597,7 +1603,7 @@
     </x:row>
     <x:row r="3" spans="1:6">
       <x:c r="A3" s="0">
-        <x:v>2</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>120</x:v>
@@ -1617,7 +1623,7 @@
     </x:row>
     <x:row r="4" spans="1:6">
       <x:c r="A4" s="0">
-        <x:v>3</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>123</x:v>
@@ -1637,7 +1643,7 @@
     </x:row>
     <x:row r="5" spans="1:6">
       <x:c r="A5" s="0">
-        <x:v>4</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>126</x:v>
@@ -1657,7 +1663,7 @@
     </x:row>
     <x:row r="6" spans="1:6">
       <x:c r="A6" s="0">
-        <x:v>5</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>129</x:v>
@@ -1677,7 +1683,7 @@
     </x:row>
     <x:row r="7" spans="1:6">
       <x:c r="A7" s="0">
-        <x:v>6</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>132</x:v>
@@ -1791,7 +1797,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="H2" s="0">
-        <x:v>120</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
         <x:v>123</x:v>
@@ -1800,7 +1806,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="K2" s="0">
-        <x:v>215</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="L2" s="0" t="s">
         <x:v>151</x:v>
@@ -1876,13 +1882,13 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="I4" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="J4" s="0">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K4" s="0">
-        <x:v>80</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="L4" s="0" t="s">
         <x:v>151</x:v>
@@ -2028,7 +2034,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F7"/>
+  <x:dimension ref="A1:F9"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="2.710625" style="0" customWidth="1"/>
@@ -2081,101 +2087,141 @@
     </x:row>
     <x:row r="3" spans="1:6">
       <x:c r="A3" s="0">
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B3" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>155</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>129</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>24</x:v>
+        <x:v>125</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
       <x:c r="A4" s="0">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B4" s="0">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>159</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>0</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:6">
       <x:c r="A5" s="0">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B5" s="0">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>162</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E5" s="0">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>75</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:6">
       <x:c r="A6" s="0">
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B6" s="0">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>165</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>0</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:6">
       <x:c r="A7" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="E7" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F7" s="0">
+        <x:v>75</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:6">
+      <x:c r="A8" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B8" s="0">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B7" s="0">
+      <x:c r="C8" s="0" t="s">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="E8" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="0">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:6">
+      <x:c r="A9" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="0">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="C7" s="0" t="s">
+      <x:c r="C9" s="0" t="s">
         <x:v>169</x:v>
       </x:c>
-      <x:c r="D7" s="0" t="s">
+      <x:c r="D9" s="0" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="E7" s="0">
+      <x:c r="E9" s="0">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F7" s="0">
+      <x:c r="F9" s="0">
         <x:v>42</x:v>
       </x:c>
     </x:row>

</xml_diff>